<commit_message>
docs: replace named samples with a single generic demo
</commit_message>
<xml_diff>
--- a/examples/recipients.xlsx
+++ b/examples/recipients.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipients" sheetId="1" r:id="R2a2be9037852415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipients" sheetId="1" r:id="Rbc6e366964da4230"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -305,106 +305,23 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="1" t="str">
-        <x:v>Aisha Khan</x:v>
+        <x:v>Demo Name</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
+        <x:v>Demo Course</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
-        <x:v>00001</x:v>
+        <x:v>DEMO-001</x:v>
       </x:c>
       <x:c r="D2" s="1" t="str">
         <x:v>6 October 2026</x:v>
       </x:c>
       <x:c r="E2" s="1" t="str">
-        <x:v>aisha@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="27" customHeight="1">
-      <x:c r="A3" s="1" t="str">
-        <x:v>Rahul Sharma</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
-      </x:c>
-      <x:c r="C3" s="4" t="str">
-        <x:v>00002</x:v>
-      </x:c>
-      <x:c r="D3" s="1" t="str">
-        <x:v>6 October 2026</x:v>
-      </x:c>
-      <x:c r="E3" s="1" t="str">
-        <x:v>rahul@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="27" customHeight="1">
-      <x:c r="A4" s="1" t="str">
-        <x:v>Meera Patel</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="str">
-        <x:v>00003</x:v>
-      </x:c>
-      <x:c r="D4" s="1" t="str">
-        <x:v>6 October 2026</x:v>
-      </x:c>
-      <x:c r="E4" s="1" t="str">
-        <x:v>meera@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="27" customHeight="1">
-      <x:c r="A5" s="1" t="str">
-        <x:v>Alexander Christopher Montgomery</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="str">
-        <x:v>00004</x:v>
-      </x:c>
-      <x:c r="D5" s="1" t="str">
-        <x:v>6 October 2026</x:v>
-      </x:c>
-      <x:c r="E5" s="1" t="str">
-        <x:v>alex@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="27" customHeight="1">
-      <x:c r="A6" s="1" t="str">
-        <x:v>Sofia Williams</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
-      </x:c>
-      <x:c r="C6" s="4" t="str">
-        <x:v>00005</x:v>
-      </x:c>
-      <x:c r="D6" s="1" t="str">
-        <x:v>6 October 2026</x:v>
-      </x:c>
-      <x:c r="E6" s="1" t="str">
-        <x:v>sofia@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="1"/>
-      <x:c r="B7" s="1" t="str">
-        <x:v>Introduction to Python</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="str">
-        <x:v>00006</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="str">
-        <x:v>6 October 2026</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="str">
-        <x:v>invalid@example.com</x:v>
+        <x:v>demo@example.com</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:A7">
+  <x:conditionalFormatting sqref="A2:A2">
     <x:cfRule type="containsBlanks" dxfId="0" priority="1"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>